<commit_message>
Remove last per-100g mentions from the workbook
Four strings survived the sweep: two sheet subtitles, a calculator target
label and a caveat note. Rewritten to price per pack.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S43qfNWsuJW5qq3LBFwnWv
</commit_message>
<xml_diff>
--- a/rte-rice-analysis/RTE_Rice_Benchmark.xlsx
+++ b/rte-rice-analysis/RTE_Rice_Benchmark.xlsx
@@ -2009,7 +2009,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Розподіл 84 позицій. грн/100 г = медіана ціни формату / медіану ваги формату.</t>
+          <t>Розподіл 84 позицій за типом паковання. Ціна — роздріб за одну упаковку.</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4877,7 @@
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>4. Найдешевший грам — смуга 200–249 г: 50 грн за 100 г, мінімум по всіх вагах.</t>
+          <t>4. Чаша — єдиний формат, присутній у шести вагових смугах із семи.</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Ben's Original медіана 41 грн/100 г при 240 г</t>
+          <t>Рівень медіани Ben's Original — 90 грн за упаковку</t>
         </is>
       </c>
       <c r="C18" s="55">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="C6" s="65" t="inlineStr">
         <is>
-          <t>Картки продавців. 2 позиції без маси виключено з грн/100 г</t>
+          <t>Картки продавців. 2 позиції без указаної маси (Trek'n Eat)</t>
         </is>
       </c>
       <c r="D6" s="66" t="inlineStr">

</xml_diff>